<commit_message>
feat(georsclip): sync fresh 6-band GeoRSCLIP conformal evaluation results
- Synced conformal_reports_all_models.xlsx (19-sheet Excel workbook)
- Synced summary_metrics.csv, per_class_coverage.csv, and run_config.json
- GeoRSCLIP_TextHead achieved 95.08% SplitCP empirical coverage and 99.77% RAPS coverage

Co-authored-by: Claude <claude@anthropic.com>
</commit_message>
<xml_diff>
--- a/Classification/georsclip/results/uncertainty_results/conformal_reports_all_models.xlsx
+++ b/Classification/georsclip/results/uncertainty_results/conformal_reports_all_models.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="92">
   <si>
     <t>model_name</t>
   </si>
@@ -135,22 +135,19 @@
     <t>timestamp_utc</t>
   </si>
   <si>
-    <t>/content/drive/My Drive/Classification/data/data.csv</t>
-  </si>
-  <si>
-    <t>/content/drive/My Drive/Classification/data/ref.csv</t>
-  </si>
-  <si>
-    <t>/content/drive/My Drive/Classification/georsclip/models</t>
-  </si>
-  <si>
-    <t>/content/drive/My Drive/Classification/georsclip/results/uncertainty_results</t>
-  </si>
-  <si>
-    <t>/content/drive/My Drive/Classification/georsclip/results</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:40:18.923939+00:00</t>
+    <t>/kaggle/input/datasets/daneshselwal/dias-6-bands-data/k001.csv</t>
+  </si>
+  <si>
+    <t>/kaggle/input/datasets/daneshselwal/dias-6-bands-data/k002.csv</t>
+  </si>
+  <si>
+    <t>/kaggle/input</t>
+  </si>
+  <si>
+    <t>/kaggle/working/Classification/georsclip/results/uncertainty_results</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:14:18.956608+00:00</t>
   </si>
   <si>
     <t>SplitConformal - GeoRSCLIP_TextHead</t>
@@ -1546,28 +1543,28 @@
         <v>0.95</v>
       </c>
       <c r="D2">
-        <v>0.9610208816705337</v>
+        <v>0.9554524361948956</v>
       </c>
       <c r="E2">
-        <v>0.9610208816705337</v>
+        <v>0.9554524361948956</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2">
-        <v>0.9610208816705337</v>
+        <v>0.9554524361948956</v>
       </c>
       <c r="H2">
-        <v>0.03897911832946636</v>
+        <v>0.04454756380510441</v>
       </c>
       <c r="I2">
-        <v>2.478602593000005</v>
+        <v>1.635503484000026</v>
       </c>
       <c r="J2">
         <v>0.05</v>
       </c>
       <c r="M2">
-        <v>0.9709816110340864</v>
+        <v>0.9671442654779449</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1581,22 +1578,22 @@
         <v>0.95</v>
       </c>
       <c r="D3">
-        <v>0.9591647331786542</v>
+        <v>0.9535962877030162</v>
       </c>
       <c r="E3">
-        <v>0.9591647331786542</v>
+        <v>0.9535962877030162</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3">
-        <v>0.9591647331786542</v>
+        <v>0.9535962877030162</v>
       </c>
       <c r="H3">
-        <v>0.04083526682134571</v>
+        <v>0.04640371229698376</v>
       </c>
       <c r="I3">
-        <v>6.160086267999986</v>
+        <v>6.024640882999961</v>
       </c>
       <c r="J3">
         <v>0.05</v>
@@ -1605,7 +1602,7 @@
         <v>4</v>
       </c>
       <c r="M3">
-        <v>0.9608362405539844</v>
+        <v>0.9606683598355508</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1619,7 +1616,7 @@
         <v>0.95</v>
       </c>
       <c r="D4">
-        <v>0.997215777262181</v>
+        <v>0.9976798143851509</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -1634,7 +1631,7 @@
         <v>0</v>
       </c>
       <c r="I4">
-        <v>0.3966462960000001</v>
+        <v>0.4198191780000116</v>
       </c>
       <c r="J4">
         <v>0.05</v>
@@ -1643,7 +1640,7 @@
         <v>0.01</v>
       </c>
       <c r="M4">
-        <v>0.9964851541648594</v>
+        <v>0.9973165260923846</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1657,28 +1654,28 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9675174013921114</v>
+        <v>0.9651972157772621</v>
       </c>
       <c r="E5">
-        <v>0.9675174013921114</v>
+        <v>0.9651972157772621</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.9675174013921114</v>
+        <v>0.9651972157772621</v>
       </c>
       <c r="H5">
-        <v>0.03248259860788863</v>
+        <v>0.03480278422273782</v>
       </c>
       <c r="I5">
-        <v>1.894464785999986</v>
+        <v>1.89956652799998</v>
       </c>
       <c r="J5">
         <v>0.05</v>
       </c>
       <c r="M5">
-        <v>0.976966138134765</v>
+        <v>0.9769042888312579</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1692,28 +1689,28 @@
         <v>0.95</v>
       </c>
       <c r="D6">
-        <v>0.9619489559164733</v>
+        <v>0.9508120649651972</v>
       </c>
       <c r="E6">
-        <v>0.9619489559164733</v>
+        <v>0.9508120649651972</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
       <c r="G6">
-        <v>0.9619489559164733</v>
+        <v>0.9508120649651972</v>
       </c>
       <c r="H6">
-        <v>0.03805104408352668</v>
+        <v>0.04918793503480278</v>
       </c>
       <c r="I6">
-        <v>2.054084757999988</v>
+        <v>1.801946968999971</v>
       </c>
       <c r="J6">
         <v>0.05</v>
       </c>
       <c r="M6">
-        <v>0.956151574861954</v>
+        <v>0.9498744061259433</v>
       </c>
     </row>
   </sheetData>
@@ -1779,7 +1776,7 @@
         <v>26</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1875,7 +1872,7 @@
         <v>36</v>
       </c>
       <c r="B19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1890,15 +1887,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1953,44 +1950,44 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9619489559164733</v>
+        <v>0.9508120649651972</v>
       </c>
       <c r="E5">
-        <v>0.9619489559164733</v>
+        <v>0.9508120649651972</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.9619489559164733</v>
+        <v>0.9508120649651972</v>
       </c>
       <c r="H5">
-        <v>0.03805104408352668</v>
+        <v>0.04918793503480278</v>
       </c>
       <c r="I5">
-        <v>2.054084757999988</v>
+        <v>1.801946968999971</v>
       </c>
       <c r="J5">
         <v>0.05</v>
       </c>
       <c r="M5">
-        <v>0.956151574861954</v>
+        <v>0.9498744061259433</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1998,7 +1995,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9824945295404814</v>
+        <v>0.9660831509846827</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -2009,7 +2006,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9493392070484582</v>
+        <v>0.9625550660792952</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -2020,7 +2017,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.9301675977653632</v>
+        <v>0.8854748603351955</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -2031,7 +2028,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>0.9487179487179487</v>
+        <v>0.967948717948718</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -2042,7 +2039,7 @@
         <v>4</v>
       </c>
       <c r="B14">
-        <v>0.9807692307692307</v>
+        <v>0.9903846153846154</v>
       </c>
       <c r="C14">
         <v>104</v>
@@ -2053,7 +2050,7 @@
         <v>5</v>
       </c>
       <c r="B15">
-        <v>0.9603960396039604</v>
+        <v>0.9207920792079208</v>
       </c>
       <c r="C15">
         <v>101</v>
@@ -2064,7 +2061,7 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>0.9411764705882353</v>
+        <v>0.9558823529411765</v>
       </c>
       <c r="C16">
         <v>68</v>
@@ -2072,18 +2069,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -2091,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C21">
-        <v>34161</v>
+        <v>33360</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -2102,10 +2099,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C22">
-        <v>11217</v>
+        <v>13130</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -2113,10 +2110,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C23">
-        <v>11732</v>
+        <v>10273</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -2124,10 +2121,10 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C24">
-        <v>3505</v>
+        <v>3796</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -2135,13 +2132,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C25">
-        <v>3182</v>
+        <v>2873</v>
       </c>
       <c r="J25" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -2149,10 +2146,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C26">
-        <v>3739</v>
+        <v>3312</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -2160,10 +2157,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C27">
-        <v>1913</v>
+        <v>1816</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -2171,35 +2168,35 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C28">
-        <v>31861</v>
+        <v>32750</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33">
-        <v>0.0365523601086174</v>
+        <v>0.03693484942004033</v>
       </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2215,15 +2212,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -2278,44 +2275,44 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9610208816705337</v>
+        <v>0.9554524361948956</v>
       </c>
       <c r="E5">
-        <v>0.9610208816705337</v>
+        <v>0.9554524361948956</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.9610208816705337</v>
+        <v>0.9554524361948956</v>
       </c>
       <c r="H5">
-        <v>0.03897911832946636</v>
+        <v>0.04454756380510441</v>
       </c>
       <c r="I5">
-        <v>2.478602593000005</v>
+        <v>1.635503484000026</v>
       </c>
       <c r="J5">
         <v>0.05</v>
       </c>
       <c r="M5">
-        <v>0.9709816110340864</v>
+        <v>0.9671442654779449</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -2323,7 +2320,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9540481400437637</v>
+        <v>0.9452954048140044</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -2334,7 +2331,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9647577092511013</v>
+        <v>0.9581497797356828</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -2356,7 +2353,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>0.9871794871794872</v>
+        <v>0.9807692307692307</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -2367,7 +2364,7 @@
         <v>4</v>
       </c>
       <c r="B14">
-        <v>0.9807692307692307</v>
+        <v>0.9903846153846154</v>
       </c>
       <c r="C14">
         <v>104</v>
@@ -2389,7 +2386,7 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>1</v>
+        <v>0.9852941176470589</v>
       </c>
       <c r="C16">
         <v>68</v>
@@ -2397,18 +2394,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -2416,10 +2413,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C21">
-        <v>32372</v>
+        <v>32063</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -2427,10 +2424,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C22">
-        <v>12824</v>
+        <v>12823</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -2438,10 +2435,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C23">
-        <v>12987</v>
+        <v>13155</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -2449,10 +2446,10 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C24">
-        <v>5180</v>
+        <v>3979</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -2460,13 +2457,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C25">
-        <v>2948</v>
+        <v>3392</v>
       </c>
       <c r="J25" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -2474,10 +2471,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C26">
-        <v>3770</v>
+        <v>3867</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -2485,10 +2482,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C27">
-        <v>2712</v>
+        <v>2301</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -2496,23 +2493,23 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C28">
-        <v>28517</v>
+        <v>29730</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -2520,7 +2517,7 @@
         <v>0</v>
       </c>
       <c r="B33">
-        <v>0.03620722189964365</v>
+        <v>0.03682234863272171</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -2528,7 +2525,7 @@
         <v>1</v>
       </c>
       <c r="B34">
-        <v>0.03959408980053603</v>
+        <v>0.03653536208164476</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -2536,7 +2533,7 @@
         <v>2</v>
       </c>
       <c r="B35">
-        <v>0.03854419496326833</v>
+        <v>0.04160375984803055</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -2544,7 +2541,7 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>0.05489601377116116</v>
+        <v>0.03783390530072506</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -2552,7 +2549,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>0.03488322404257749</v>
+        <v>0.05456513562654786</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -2560,7 +2557,7 @@
         <v>5</v>
       </c>
       <c r="B38">
-        <v>0.03696727640573783</v>
+        <v>0.04249608324117005</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -2568,17 +2565,17 @@
         <v>6</v>
       </c>
       <c r="B39">
-        <v>0.3533661612421157</v>
+        <v>0.07954848886864618</v>
       </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2594,15 +2591,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -2657,44 +2654,44 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9675174013921114</v>
+        <v>0.9651972157772621</v>
       </c>
       <c r="E5">
-        <v>0.9675174013921114</v>
+        <v>0.9651972157772621</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.9675174013921114</v>
+        <v>0.9651972157772621</v>
       </c>
       <c r="H5">
-        <v>0.03248259860788863</v>
+        <v>0.03480278422273782</v>
       </c>
       <c r="I5">
-        <v>1.894464785999986</v>
+        <v>1.89956652799998</v>
       </c>
       <c r="J5">
         <v>0.05</v>
       </c>
       <c r="M5">
-        <v>0.976966138134765</v>
+        <v>0.9769042888312579</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -2702,7 +2699,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9595185995623632</v>
+        <v>0.9518599562363238</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -2713,7 +2710,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.973568281938326</v>
+        <v>0.9625550660792952</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -2724,7 +2721,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.9581005586592178</v>
+        <v>0.9776536312849162</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -2735,7 +2732,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>0.9871794871794872</v>
+        <v>0.9807692307692307</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -2757,7 +2754,7 @@
         <v>5</v>
       </c>
       <c r="B15">
-        <v>0.9603960396039604</v>
+        <v>0.9801980198019802</v>
       </c>
       <c r="C15">
         <v>101</v>
@@ -2768,7 +2765,7 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>1</v>
+        <v>0.9852941176470589</v>
       </c>
       <c r="C16">
         <v>68</v>
@@ -2776,18 +2773,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -2795,10 +2792,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C21">
-        <v>32668</v>
+        <v>32256</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -2806,10 +2803,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C22">
-        <v>13293</v>
+        <v>12992</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -2817,10 +2814,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C23">
-        <v>13413</v>
+        <v>14023</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -2828,10 +2825,10 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C24">
-        <v>5259</v>
+        <v>4353</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -2839,13 +2836,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C25">
-        <v>3742</v>
+        <v>4468</v>
       </c>
       <c r="J25" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -2853,10 +2850,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C26">
-        <v>4233</v>
+        <v>4650</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -2864,10 +2861,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C27">
-        <v>2712</v>
+        <v>2301</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -2875,26 +2872,26 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C28">
-        <v>25990</v>
+        <v>26267</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -2902,7 +2899,7 @@
         <v>0</v>
       </c>
       <c r="B33">
-        <v>0.03624211028097235</v>
+        <v>0.03683457261218759</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -2913,7 +2910,7 @@
         <v>1</v>
       </c>
       <c r="B34">
-        <v>0.04154661068893084</v>
+        <v>0.03675291046515261</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -2924,7 +2921,7 @@
         <v>2</v>
       </c>
       <c r="B35">
-        <v>0.03971777142198163</v>
+        <v>0.04677543506683224</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -2935,7 +2932,7 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>0.05687480901426112</v>
+        <v>0.04062399567916974</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -2946,7 +2943,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>0.05420263052844188</v>
+        <v>0.4609798571989133</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -2957,7 +2954,7 @@
         <v>5</v>
       </c>
       <c r="B38">
-        <v>0.04389244857789132</v>
+        <v>0.06558514946029104</v>
       </c>
       <c r="C38">
         <v>1</v>
@@ -2968,7 +2965,7 @@
         <v>6</v>
       </c>
       <c r="B39">
-        <v>0.3533661612421157</v>
+        <v>0.07954848886864618</v>
       </c>
       <c r="C39">
         <v>1</v>
@@ -2976,12 +2973,12 @@
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2997,15 +2994,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -3060,22 +3057,22 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9591647331786542</v>
+        <v>0.9535962877030162</v>
       </c>
       <c r="E5">
-        <v>0.9591647331786542</v>
+        <v>0.9535962877030162</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.9591647331786542</v>
+        <v>0.9535962877030162</v>
       </c>
       <c r="H5">
-        <v>0.04083526682134571</v>
+        <v>0.04640371229698376</v>
       </c>
       <c r="I5">
-        <v>6.160086267999986</v>
+        <v>6.024640882999961</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -3084,23 +3081,23 @@
         <v>4</v>
       </c>
       <c r="M5">
-        <v>0.9608362405539844</v>
+        <v>0.9606683598355508</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -3108,7 +3105,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9660831509846827</v>
+        <v>0.9442013129102844</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -3119,7 +3116,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9405286343612335</v>
+        <v>0.9625550660792952</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -3141,7 +3138,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>0.9871794871794872</v>
+        <v>0.9615384615384616</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -3152,7 +3149,7 @@
         <v>4</v>
       </c>
       <c r="B14">
-        <v>0.9807692307692307</v>
+        <v>0.9903846153846154</v>
       </c>
       <c r="C14">
         <v>104</v>
@@ -3174,7 +3171,7 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>0.9411764705882353</v>
+        <v>0.9558823529411765</v>
       </c>
       <c r="C16">
         <v>68</v>
@@ -3182,15 +3179,15 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -3198,7 +3195,7 @@
         <v>0</v>
       </c>
       <c r="B21">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -3206,7 +3203,7 @@
         <v>1</v>
       </c>
       <c r="B22">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -3214,7 +3211,7 @@
         <v>2</v>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -3222,7 +3219,7 @@
         <v>3</v>
       </c>
       <c r="B24">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -3230,10 +3227,10 @@
         <v>4</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J25" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -3241,7 +3238,7 @@
         <v>5</v>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -3249,20 +3246,20 @@
         <v>6</v>
       </c>
       <c r="B27">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -3270,7 +3267,7 @@
         <v>0</v>
       </c>
       <c r="B32">
-        <v>0.03772099124696082</v>
+        <v>0.04160375984803055</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -3278,7 +3275,7 @@
         <v>1</v>
       </c>
       <c r="B33">
-        <v>0.03628068623848646</v>
+        <v>0.04249608324117005</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -3286,7 +3283,7 @@
         <v>2</v>
       </c>
       <c r="B34">
-        <v>0.03854419496326833</v>
+        <v>0.03681600362952053</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -3294,20 +3291,20 @@
         <v>3</v>
       </c>
       <c r="B35">
-        <v>0.05489601377116116</v>
+        <v>0.03849247789178822</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -3315,7 +3312,7 @@
         <v>0</v>
       </c>
       <c r="B40">
-        <v>0.9669117647058824</v>
+        <v>0.9523809523809523</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -3323,7 +3320,7 @@
         <v>1</v>
       </c>
       <c r="B41">
-        <v>0.9569028487947406</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -3331,7 +3328,7 @@
         <v>2</v>
       </c>
       <c r="B42">
-        <v>0.947075208913649</v>
+        <v>0.9501965923984272</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -3339,20 +3336,20 @@
         <v>3</v>
       </c>
       <c r="B43">
-        <v>0.9935483870967742</v>
+        <v>0.9767441860465116</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -3360,7 +3357,7 @@
         <v>0</v>
       </c>
       <c r="B48">
-        <v>0.9650273224043716</v>
+        <v>0.9452354874041621</v>
       </c>
     </row>
     <row r="49" spans="1:10">
@@ -3368,10 +3365,10 @@
         <v>1</v>
       </c>
       <c r="B49">
-        <v>0.9405286343612335</v>
+        <v>0.9583333333333334</v>
       </c>
       <c r="J49" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -3379,7 +3376,7 @@
         <v>2</v>
       </c>
       <c r="B50">
-        <v>0.947075208913649</v>
+        <v>0.9523809523809523</v>
       </c>
     </row>
     <row r="51" spans="1:10">
@@ -3387,7 +3384,7 @@
         <v>3</v>
       </c>
       <c r="B51">
-        <v>0.9935483870967742</v>
+        <v>0.9554140127388535</v>
       </c>
     </row>
     <row r="52" spans="1:10">
@@ -3395,7 +3392,7 @@
         <v>4</v>
       </c>
       <c r="B52">
-        <v>0.9807692307692307</v>
+        <v>0.9903846153846154</v>
       </c>
     </row>
     <row r="53" spans="1:10">
@@ -3411,12 +3408,12 @@
         <v>6</v>
       </c>
       <c r="B54">
-        <v>0.9411764705882353</v>
+        <v>0.9558823529411765</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -3432,15 +3429,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -3495,7 +3492,7 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.997215777262181</v>
+        <v>0.9976798143851509</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -3510,7 +3507,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>0.3966462960000001</v>
+        <v>0.4198191780000116</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -3519,23 +3516,23 @@
         <v>0.01</v>
       </c>
       <c r="M5">
-        <v>0.9964851541648594</v>
+        <v>0.9973165260923846</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -3554,7 +3551,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9955947136563876</v>
+        <v>0.9977973568281938</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -3565,7 +3562,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.9972067039106145</v>
+        <v>0.994413407821229</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -3576,7 +3573,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>0.9935897435897436</v>
+        <v>1</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -3617,18 +3614,18 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -3655,7 +3652,7 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -3710,41 +3707,41 @@
         <v>0.95</v>
       </c>
       <c r="D4">
-        <v>0.9591647331786542</v>
+        <v>0.9535962877030162</v>
       </c>
       <c r="E4">
-        <v>0.9591647331786542</v>
+        <v>0.9535962877030162</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4">
-        <v>0.9591647331786542</v>
+        <v>0.9535962877030162</v>
       </c>
       <c r="H4">
-        <v>0.04083526682134571</v>
+        <v>0.04640371229698376</v>
       </c>
       <c r="I4" t="s">
         <v>13</v>
       </c>
       <c r="J4">
-        <v>0.9608362405539844</v>
+        <v>0.9606683598355507</v>
       </c>
       <c r="L4">
         <v>4</v>
       </c>
       <c r="M4">
-        <v>0.9608362405539844</v>
+        <v>0.9606683598355508</v>
       </c>
     </row>
     <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -3760,7 +3757,7 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -3815,7 +3812,7 @@
         <v>0.95</v>
       </c>
       <c r="D4">
-        <v>0.997215777262181</v>
+        <v>0.9976798143851509</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -3833,23 +3830,23 @@
         <v>13</v>
       </c>
       <c r="J4">
-        <v>0.9964851541648594</v>
+        <v>0.9973165260923847</v>
       </c>
       <c r="K4">
         <v>0.01</v>
       </c>
       <c r="M4">
-        <v>0.9964851541648594</v>
+        <v>0.9973165260923846</v>
       </c>
     </row>
     <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>